<commit_message>
sync: update stable cost analysis and round2 outputs
</commit_message>
<xml_diff>
--- a/outputs/stable_cost_prompt_iteration/stable_cost_summary.xlsx
+++ b/outputs/stable_cost_prompt_iteration/stable_cost_summary.xlsx
@@ -428,7 +428,7 @@
   <dimension ref="A1:T8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
     <col width="33" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -555,7 +555,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Condition 3</t>
+          <t>R1-P3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -603,7 +603,7 @@
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0977</v>
+        <v>0.0961</v>
       </c>
       <c r="Q2" t="n">
         <v>1</v>
@@ -627,7 +627,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Condition 7</t>
+          <t>R1-P7</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -672,10 +672,10 @@
         <v>0.35</v>
       </c>
       <c r="O3" t="n">
-        <v>0.0109</v>
+        <v>0.0328</v>
       </c>
       <c r="P3" t="n">
-        <v>0.1387</v>
+        <v>0.1456</v>
       </c>
       <c r="Q3" t="n">
         <v>2</v>
@@ -699,7 +699,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Condition 4</t>
+          <t>R1-P4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -747,7 +747,7 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>0.1499</v>
+        <v>0.1524</v>
       </c>
       <c r="Q4" t="n">
         <v>3</v>
@@ -771,7 +771,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Condition 2</t>
+          <t>R1-P2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -816,10 +816,10 @@
         <v>0.358</v>
       </c>
       <c r="O5" t="n">
-        <v>0.0019</v>
+        <v>0.0056</v>
       </c>
       <c r="P5" t="n">
-        <v>0.1721</v>
+        <v>0.1656</v>
       </c>
       <c r="Q5" t="n">
         <v>4</v>
@@ -843,7 +843,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Condition 1</t>
+          <t>R1-P1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -888,10 +888,10 @@
         <v>0.738</v>
       </c>
       <c r="O6" t="n">
-        <v>0.0545</v>
+        <v>0.1636</v>
       </c>
       <c r="P6" t="n">
-        <v>0.2827</v>
+        <v>0.3172</v>
       </c>
       <c r="Q6" t="n">
         <v>5</v>
@@ -915,7 +915,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Condition 5</t>
+          <t>R1-P5</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -960,10 +960,10 @@
         <v>0.82</v>
       </c>
       <c r="O7" t="n">
-        <v>0.1072</v>
+        <v>0.3216</v>
       </c>
       <c r="P7" t="n">
-        <v>0.3085</v>
+        <v>0.378</v>
       </c>
       <c r="Q7" t="n">
         <v>6</v>
@@ -987,7 +987,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Condition 6</t>
+          <t>R1-P6</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1032,10 +1032,10 @@
         <v>0.98</v>
       </c>
       <c r="O8" t="n">
-        <v>0.1357</v>
+        <v>0.4072</v>
       </c>
       <c r="P8" t="n">
-        <v>0.3518</v>
+        <v>0.4399</v>
       </c>
       <c r="Q8" t="n">
         <v>7</v>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>C_norm: Responses are not close enough to full-score target</t>
+          <t>C_weak: One dimension is underdeveloped; weakest dimension: D1</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">

</xml_diff>